<commit_message>
Fix note-numbering row in spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Divergencias_DN700_022-007300.xlsx
+++ b/Divergencias_DN700_022-007300.xlsx
@@ -1346,12 +1346,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>007343, 007344, 007350, 007301</t>
+          <t>007343, 007344, 007350</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Numeração das notas repetida (item "2" duas vezes; 007301 sem nota 2 nas 007304/05/06 etc.).</t>
+          <t>Numeração das notas repetida (item "2" aparece duas vezes, faltando o 3).</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">

</xml_diff>